<commit_message>
added more stuff to the BOM
</commit_message>
<xml_diff>
--- a/hardware/bom/bom.xlsx
+++ b/hardware/bom/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hellc\OneDrive\Documentos\altoidometer\hardware\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1A1787-8F37-46E4-8A86-42E20A84D94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765087C1-B483-4C73-82A1-F913205E1FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>Part</t>
   </si>
@@ -63,9 +63,6 @@
     <t>22k</t>
   </si>
   <si>
-    <t>MAX42248</t>
-  </si>
-  <si>
     <t>Part Name</t>
   </si>
   <si>
@@ -148,6 +145,63 @@
   </si>
   <si>
     <t>for the SOIC-8 to DIP-8 adapter, not needed for PCB</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/AITRIP-ESP-WROOM-32-Development-Microcontroller-Integrated/dp/B0CR5Y2JVD?crid=1N580DYU2QSZ7&amp;dib=eyJ2IjoiMSJ9.nnu8chisPogby2CLqTPsn5F7JgjX13u6rdbmtL8t2c8lpjmEcdGuLD3w7BvVDTRtelHrpY2e0VmQL8K5cgI3a4jTMxUUzwKf54fgRpCS1fGv4JG8_9DWqFHioOA7b2XyX7HvoE2sm7GQcrTHo9J6sY1jNA38CYL7jNuJKW4oBLFmn8rMWLLlYb7iY_GsiOxf6pFqVNfMwE4MUytw4uB3klFSjNz3p9r08ZNmrAc-Zd8.s5V8F1nHPfwIpT37nUKmS7hFquENuqdEL7cb3Oiy3hw&amp;dib_tag=se&amp;keywords=esp32%2Bdevkit%2Bv1%2Btype%2Bc&amp;qid=1786237513&amp;sprefix=esp32%2Bdevkit%2Bv1%2Btype%2B%2Caps%2C141&amp;sr=8-4&amp;th=1</t>
+  </si>
+  <si>
+    <t>ESP32 Devkit V1 Type-C</t>
+  </si>
+  <si>
+    <t>1 needed, link is for a pack of 3 cus ur def gonna fry at least one</t>
+  </si>
+  <si>
+    <t>Double-sided perfboard</t>
+  </si>
+  <si>
+    <t>2 needed, links is for a 5 pack</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Double-Sided-Universal-Packs-12x18/dp/B08WJBS4HK?crid=1AOR6VFVJKBA8&amp;dib=eyJ2IjoiMSJ9.IJZxxF3y-NAmxVI1-19qUG7FdbCXY0AhMIsTbbRJ6BSAYS8fiMepjsX24L2cz8P10Owr0-HJD2iY9gLvIO05LCxJ5T5K4pM30dZIq3qLyebKALfUhq7-ckMHsDdmBbnp-teyfvkuRz4cJdJ7RkbK8-mew1YjB6UhxuU4tFEzk8l3XiDwaUwZY-IMiUC2O6GoGPp62hL7wbEXUpJ3hyFA4xvz3xp0k2ETLrlLTUJdFGM.JztVQ17eEOgjFlCnVPcLhTmZtq32tNcnibzp1Mqz3wI&amp;dib_tag=se&amp;keywords=perfboard&amp;qid=1786237816&amp;sprefix=perfboard%2Caps%2C153&amp;sr=8-10</t>
+  </si>
+  <si>
+    <t>Altoids tin</t>
+  </si>
+  <si>
+    <t>flavour doesn’t matter, u gotta eat the mints first</t>
+  </si>
+  <si>
+    <t>just go to the store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAX44248ASA+ </t>
+  </si>
+  <si>
+    <t>this one is discontinued so find something similar if its not in stock</t>
+  </si>
+  <si>
+    <t>4mm Banana jack</t>
+  </si>
+  <si>
+    <t>https://www.adafruit.com/product/3691</t>
+  </si>
+  <si>
+    <t>SJ3-35063A</t>
+  </si>
+  <si>
+    <t>3.5mm Audio jack</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/SJ3-35063A/24627956</t>
+  </si>
+  <si>
+    <t>Flexible stranded jumper wires</t>
+  </si>
+  <si>
+    <t>a bunch</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/ELEGOO-Solderless-Flexible-Breadboard-Compatible/dp/B09ZQP9LB6?crid=1P7HCMQ2RVJFK&amp;dib=eyJ2IjoiMSJ9.cLcguCO2XFnX7DP0vhpAnqUMp4CZbdFYCe5LoPu0ofBCDVuwUeYRcwPmGak_QHN5PrLY-ZdSibTVkzH9BHquMqkZq_7vSKdgHWkeOwamz6urwTdXo2PA3RgKvDeHvb0e992Tt_UQ1MMD3iH0r-lzrJ1UoDGKzeDJ9r1NKBkQqE9FTjF2VSAG07CXEm_6oqFJyr5mU9UEzVMAVpH4r2UYbjeJvyOQAq0aOJy2UkNxkkQ.QyLogNp25RM9325gYR5A282dSAriDrGSKkhVvd_Cxzs&amp;dib_tag=se&amp;keywords=flexible+male+to+male+jumper+wires&amp;qid=1786238683&amp;sprefix=flexible+male+to+male+jumper+wires%2Caps%2C150&amp;sr=8-4</t>
   </si>
 </sst>
 </file>
@@ -225,8 +279,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}" name="Table1" displayName="Table1" ref="A1:G12" totalsRowShown="0">
-  <autoFilter ref="A1:G12" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}" name="Table1" displayName="Table1" ref="A1:G42" totalsRowShown="0">
+  <autoFilter ref="A1:G42" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{E2F33036-2458-4970-9DFB-B5AAD95E2E08}" name="Part" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{0F8E33A6-EF39-42D8-BEAB-3964F6866563}" name="Part Name"/>
@@ -503,13 +557,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="54.28515625" customWidth="1"/>
+    <col min="6" max="6" width="60.140625" customWidth="1"/>
     <col min="7" max="7" width="132.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -518,7 +572,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -533,15 +587,15 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -556,15 +610,15 @@
         <v>2</v>
       </c>
       <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -579,15 +633,15 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -602,15 +656,15 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
@@ -625,15 +679,15 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
@@ -648,41 +702,41 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -690,71 +744,74 @@
       <c r="E8">
         <v>4</v>
       </c>
+      <c r="F8" t="s">
+        <v>50</v>
+      </c>
       <c r="G8" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
         <v>23</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10">
         <v>10</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
         <v>34</v>
       </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -762,22 +819,151 @@
         <v>61300811121</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>37</v>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -792,10 +978,14 @@
     <hyperlink ref="G6" r:id="rId8" xr:uid="{0199E0BE-AAB1-4C2B-BB5E-D58D9FEFA299}"/>
     <hyperlink ref="G11" r:id="rId9" xr:uid="{A7A68B94-84D8-46EB-A56E-312BCF262967}"/>
     <hyperlink ref="G12" r:id="rId10" xr:uid="{35484E0A-C766-44A6-948D-070D0EC0D422}"/>
+    <hyperlink ref="G14" r:id="rId11" display="https://www.amazon.com/Double-Sided-Universal-Packs-12x18/dp/B08WJBS4HK?crid=1AOR6VFVJKBA8&amp;dib=eyJ2IjoiMSJ9.IJZxxF3y-NAmxVI1-19qUG7FdbCXY0AhMIsTbbRJ6BSAYS8fiMepjsX24L2cz8P10Owr0-HJD2iY9gLvIO05LCxJ5T5K4pM30dZIq3qLyebKALfUhq7-ckMHsDdmBbnp-teyfvkuRz4cJdJ7RkbK8-mew1YjB6UhxuU4tFEzk8l3XiDwaUwZY-IMiUC2O6GoGPp62hL7wbEXUpJ3hyFA4xvz3xp0k2ETLrlLTUJdFGM.JztVQ17eEOgjFlCnVPcLhTmZtq32tNcnibzp1Mqz3wI&amp;dib_tag=se&amp;keywords=perfboard&amp;qid=1786237816&amp;sprefix=perfboard%2Caps%2C153&amp;sr=8-10" xr:uid="{28AE0D3F-6318-47A3-8202-C28FFDA989D1}"/>
+    <hyperlink ref="G16" r:id="rId12" xr:uid="{B8BD8862-1226-415A-B4E2-8369095C9FD8}"/>
+    <hyperlink ref="G17" r:id="rId13" xr:uid="{8B054EC8-1A8D-4FE8-81F3-777DFD36B139}"/>
+    <hyperlink ref="G18" r:id="rId14" display="https://www.amazon.com/ELEGOO-Solderless-Flexible-Breadboard-Compatible/dp/B09ZQP9LB6?crid=1P7HCMQ2RVJFK&amp;dib=eyJ2IjoiMSJ9.cLcguCO2XFnX7DP0vhpAnqUMp4CZbdFYCe5LoPu0ofBCDVuwUeYRcwPmGak_QHN5PrLY-ZdSibTVkzH9BHquMqkZq_7vSKdgHWkeOwamz6urwTdXo2PA3RgKvDeHvb0e992Tt_UQ1MMD3iH0r-lzrJ1UoDGKzeDJ9r1NKBkQqE9FTjF2VSAG07CXEm_6oqFJyr5mU9UEzVMAVpH4r2UYbjeJvyOQAq0aOJy2UkNxkkQ.QyLogNp25RM9325gYR5A282dSAriDrGSKkhVvd_Cxzs&amp;dib_tag=se&amp;keywords=flexible+male+to+male+jumper+wires&amp;qid=1786238683&amp;sprefix=flexible+male+to+male+jumper+wires%2Caps%2C150&amp;sr=8-4" xr:uid="{992AFD92-C626-47BA-B823-B6A1DC58C763}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changed audio jack configuration and added microsd card module
</commit_message>
<xml_diff>
--- a/hardware/bom/bom.xlsx
+++ b/hardware/bom/bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hellc\OneDrive\Documentos\altoidometer\hardware\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765087C1-B483-4C73-82A1-F913205E1FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942FA830-914A-40AF-BFC4-F0AEC40B8B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
   <si>
     <t>Part</t>
   </si>
@@ -202,6 +202,15 @@
   </si>
   <si>
     <t>https://www.amazon.com/ELEGOO-Solderless-Flexible-Breadboard-Compatible/dp/B09ZQP9LB6?crid=1P7HCMQ2RVJFK&amp;dib=eyJ2IjoiMSJ9.cLcguCO2XFnX7DP0vhpAnqUMp4CZbdFYCe5LoPu0ofBCDVuwUeYRcwPmGak_QHN5PrLY-ZdSibTVkzH9BHquMqkZq_7vSKdgHWkeOwamz6urwTdXo2PA3RgKvDeHvb0e992Tt_UQ1MMD3iH0r-lzrJ1UoDGKzeDJ9r1NKBkQqE9FTjF2VSAG07CXEm_6oqFJyr5mU9UEzVMAVpH4r2UYbjeJvyOQAq0aOJy2UkNxkkQ.QyLogNp25RM9325gYR5A282dSAriDrGSKkhVvd_Cxzs&amp;dib_tag=se&amp;keywords=flexible+male+to+male+jumper+wires&amp;qid=1786238683&amp;sprefix=flexible+male+to+male+jumper+wires%2Caps%2C150&amp;sr=8-4</t>
+  </si>
+  <si>
+    <t>MicroSD Card Module</t>
+  </si>
+  <si>
+    <t>get this one or any one that has the same footprint</t>
+  </si>
+  <si>
+    <t>https://protosupplies.com/product/microsd-card-module/</t>
   </si>
 </sst>
 </file>
@@ -251,8 +260,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -260,10 +269,10 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -282,13 +291,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}" name="Table1" displayName="Table1" ref="A1:G42" totalsRowShown="0">
   <autoFilter ref="A1:G42" xr:uid="{3A8F9497-97EC-48C8-A023-4CC4F33E3B74}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E2F33036-2458-4970-9DFB-B5AAD95E2E08}" name="Part" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{E2F33036-2458-4970-9DFB-B5AAD95E2E08}" name="Part" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{0F8E33A6-EF39-42D8-BEAB-3964F6866563}" name="Part Name"/>
     <tableColumn id="2" xr3:uid="{F8DC5730-0F3A-4CCE-9669-0073A1BF55B8}" name="Value"/>
     <tableColumn id="3" xr3:uid="{C19FA264-DDBF-4C46-9C91-6D65D8F11412}" name="Package"/>
     <tableColumn id="4" xr3:uid="{E59DC8FF-580C-4133-BAE2-B92C193A6F1D}" name="Qty"/>
     <tableColumn id="5" xr3:uid="{8A545747-1918-4FD2-A3E3-43540949A549}" name="Notes"/>
-    <tableColumn id="7" xr3:uid="{B998C087-71DB-4BA5-91B0-A5B38D6770A8}" name="Link" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{B998C087-71DB-4BA5-91B0-A5B38D6770A8}" name="Link" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -557,14 +566,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="60.140625" customWidth="1"/>
-    <col min="7" max="7" width="132.140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="132.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -586,7 +595,7 @@
       <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>15</v>
       </c>
       <c r="H1" t="s">
@@ -612,7 +621,7 @@
       <c r="F2" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -635,7 +644,7 @@
       <c r="F3" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -658,7 +667,7 @@
       <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -681,7 +690,7 @@
       <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -704,7 +713,7 @@
       <c r="F6" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -724,7 +733,7 @@
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -747,7 +756,7 @@
       <c r="F8" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -767,7 +776,7 @@
       <c r="E9">
         <v>1</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -787,7 +796,7 @@
       <c r="E10">
         <v>10</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -810,7 +819,7 @@
       <c r="F11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -833,7 +842,7 @@
       <c r="F12" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -856,7 +865,7 @@
       <c r="F13" t="s">
         <v>42</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -879,7 +888,7 @@
       <c r="F14" t="s">
         <v>44</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -902,7 +911,7 @@
       <c r="F15" t="s">
         <v>47</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" t="s">
         <v>48</v>
       </c>
     </row>
@@ -922,7 +931,7 @@
       <c r="E16">
         <v>3</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -942,7 +951,7 @@
       <c r="E17">
         <v>2</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -962,8 +971,31 @@
       <c r="E18" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="2" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -982,10 +1014,11 @@
     <hyperlink ref="G16" r:id="rId12" xr:uid="{B8BD8862-1226-415A-B4E2-8369095C9FD8}"/>
     <hyperlink ref="G17" r:id="rId13" xr:uid="{8B054EC8-1A8D-4FE8-81F3-777DFD36B139}"/>
     <hyperlink ref="G18" r:id="rId14" display="https://www.amazon.com/ELEGOO-Solderless-Flexible-Breadboard-Compatible/dp/B09ZQP9LB6?crid=1P7HCMQ2RVJFK&amp;dib=eyJ2IjoiMSJ9.cLcguCO2XFnX7DP0vhpAnqUMp4CZbdFYCe5LoPu0ofBCDVuwUeYRcwPmGak_QHN5PrLY-ZdSibTVkzH9BHquMqkZq_7vSKdgHWkeOwamz6urwTdXo2PA3RgKvDeHvb0e992Tt_UQ1MMD3iH0r-lzrJ1UoDGKzeDJ9r1NKBkQqE9FTjF2VSAG07CXEm_6oqFJyr5mU9UEzVMAVpH4r2UYbjeJvyOQAq0aOJy2UkNxkkQ.QyLogNp25RM9325gYR5A282dSAriDrGSKkhVvd_Cxzs&amp;dib_tag=se&amp;keywords=flexible+male+to+male+jumper+wires&amp;qid=1786238683&amp;sprefix=flexible+male+to+male+jumper+wires%2Caps%2C150&amp;sr=8-4" xr:uid="{992AFD92-C626-47BA-B823-B6A1DC58C763}"/>
+    <hyperlink ref="G19" r:id="rId15" xr:uid="{A6CDCCD5-A78D-410D-B1A8-1055CE0BB037}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix error in bom that i made -_-
</commit_message>
<xml_diff>
--- a/hardware/bom/bom.xlsx
+++ b/hardware/bom/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hellc\OneDrive\Documentos\altoidometer\hardware\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06308F43-3A8B-497A-AF88-8E958AF333DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912F732D-E79E-43DB-86B6-C358992822BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="65">
   <si>
     <t>Part</t>
   </si>
@@ -963,7 +963,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="B19" t="s">
         <v>58</v>
@@ -982,6 +982,9 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="B20" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
oops (didnt save bom)
</commit_message>
<xml_diff>
--- a/hardware/bom/bom.xlsx
+++ b/hardware/bom/bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hellc\OneDrive\Documentos\altoidometer\hardware\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912F732D-E79E-43DB-86B6-C358992822BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B778BF-E678-4545-8953-0750D460286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1455" yWindow="3375" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="72">
   <si>
     <t>Part</t>
   </si>
@@ -220,6 +220,27 @@
   </si>
   <si>
     <t>https://www.lowes.com/pd/Scotch-Super-33-0-75-in-x-37-5-ft-Vinyl-Electrical-Tape-Black/3128055</t>
+  </si>
+  <si>
+    <t>9-Axis IMU</t>
+  </si>
+  <si>
+    <t>9-DOF LSM9DS1 BREAKOUT BOARD - S</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/adafruit-industries-llc/4634/12503966</t>
+  </si>
+  <si>
+    <t>GPS Module</t>
+  </si>
+  <si>
+    <t>ULTIMATE GPS PA1616D BREAKOUT</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/adafruit-industries-llc/5440/16511257</t>
+  </si>
+  <si>
+    <t>microSD card module</t>
   </si>
 </sst>
 </file>
@@ -549,11 +570,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
     <col min="3" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="62.85546875" customWidth="1"/>
     <col min="7" max="7" width="132.140625" customWidth="1"/>
@@ -986,7 +1007,7 @@
         <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1002,6 +1023,46 @@
       </c>
       <c r="G20" s="2" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1022,11 +1083,14 @@
     <hyperlink ref="G19" r:id="rId14" display="https://www.amazon.com/ELEGOO-Solderless-Flexible-Breadboard-Compatible/dp/B09ZQP9LB6?crid=1P7HCMQ2RVJFK&amp;dib=eyJ2IjoiMSJ9.cLcguCO2XFnX7DP0vhpAnqUMp4CZbdFYCe5LoPu0ofBCDVuwUeYRcwPmGak_QHN5PrLY-ZdSibTVkzH9BHquMqkZq_7vSKdgHWkeOwamz6urwTdXo2PA3RgKvDeHvb0e992Tt_UQ1MMD3iH0r-lzrJ1UoDGKzeDJ9r1NKBkQqE9FTjF2VSAG07CXEm_6oqFJyr5mU9UEzVMAVpH4r2UYbjeJvyOQAq0aOJy2UkNxkkQ.QyLogNp25RM9325gYR5A282dSAriDrGSKkhVvd_Cxzs&amp;dib_tag=se&amp;keywords=flexible+male+to+male+jumper+wires&amp;qid=1786238683&amp;sprefix=flexible+male+to+male+jumper+wires%2Caps%2C150&amp;sr=8-4" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
     <hyperlink ref="G20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="G16" r:id="rId16" xr:uid="{732DF290-5F6F-4C0A-86A2-D02F00CE6AF1}"/>
+    <hyperlink ref="G21" r:id="rId17" xr:uid="{B3DAACF8-C198-4C4B-8275-FC1F0ACF886F}"/>
+    <hyperlink ref="G22" r:id="rId18" xr:uid="{E94F441E-82E2-4ACC-BB70-658490E52A20}"/>
+    <hyperlink ref="G2" r:id="rId19" xr:uid="{721849B8-DC69-40F8-9EA9-A49B9CD331F8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId20"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change discontinued part on BOM
</commit_message>
<xml_diff>
--- a/hardware/bom/bom.xlsx
+++ b/hardware/bom/bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hellc\OneDrive\Documentos\altoidometer\hardware\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B778BF-E678-4545-8953-0750D460286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53A501A-398C-415F-AE72-C0AC5B422A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1455" yWindow="3375" windowWidth="28800" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
   <si>
     <t>Part</t>
   </si>
@@ -105,18 +105,9 @@
     <t>https://www.mouser.com/en/ProductDetail/Analog-Devices-Maxim-Integrated/MAX44248ASA%2b?qs=NHTRUjBBRiOumtQwF0J%2F%2FA%3D%3D</t>
   </si>
   <si>
-    <t>BAT85,113</t>
-  </si>
-  <si>
     <t>Schottky diode</t>
   </si>
   <si>
-    <t>this one is discontinued so find something similar if its not in stock</t>
-  </si>
-  <si>
-    <t>https://www.rocelec.com/part/01t4w00000POnOFAA1-BAT85113</t>
-  </si>
-  <si>
     <t>DLS23028B</t>
   </si>
   <si>
@@ -241,6 +232,12 @@
   </si>
   <si>
     <t>microSD card module</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-general-semiconductor-diodes-division/BAT85S-TAP/3104127</t>
+  </si>
+  <si>
+    <t>BAT85S-TAP</t>
   </si>
 </sst>
 </file>
@@ -743,10 +740,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
         <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
@@ -757,19 +754,16 @@
       <c r="E8">
         <v>4</v>
       </c>
-      <c r="F8" t="s">
-        <v>28</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -781,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -789,7 +783,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
@@ -801,30 +795,30 @@
         <v>10</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -832,7 +826,7 @@
         <v>61300811121</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
@@ -844,10 +838,10 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -855,7 +849,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -867,10 +861,10 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -878,7 +872,7 @@
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
@@ -890,10 +884,10 @@
         <v>2</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -901,7 +895,7 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
@@ -913,10 +907,10 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -924,7 +918,7 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
@@ -936,18 +930,18 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
@@ -959,7 +953,7 @@
         <v>3</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,7 +961,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C18" t="s">
         <v>8</v>
@@ -979,7 +973,7 @@
         <v>2</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -987,7 +981,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
@@ -996,18 +990,18 @@
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1019,18 +1013,18 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C21" t="s">
         <v>8</v>
@@ -1042,15 +1036,15 @@
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1062,7 +1056,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>